<commit_message>
Primera versión estable para la limpieza de datos
</commit_message>
<xml_diff>
--- a/Data-Analytics/docs/FLEX DRIVE - Permítenos Conocerte.xlsx
+++ b/Data-Analytics/docs/FLEX DRIVE - Permítenos Conocerte.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leshi\OneDrive\Escritorio\University\006- Ninth Semester\000- Flex Drive\Flex-Drive\Data-Analytics\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\7SEMESTRE\FlexDrive\big data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC9A6E2-7D7C-4AF7-AC7C-1E6128C938B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE7762F7-991D-4111-844D-87249F76B51F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -4777,96 +4777,96 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CI384"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="104" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="90.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="90.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="38" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="137.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="73.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="137.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="73.109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="70" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="40.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="125.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="67.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="59.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="125.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="67.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="18" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="240.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="72.42578125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="217.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="223.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="35.85546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="96.5703125" bestFit="1" customWidth="1"/>
-    <col min="33" max="34" width="255.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="240.109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="72.44140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="217.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="223.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="35.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="96.5546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="255.6640625" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="44" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="113" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="39.42578125" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="50.7109375" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="49.85546875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="50.6640625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="49.88671875" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="51" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="37.85546875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="38.5703125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="38.140625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="240.28515625" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="132.42578125" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="116.7109375" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="47.5703125" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="44.28515625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="44.5703125" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="55.7109375" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="39.28515625" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="129.28515625" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="155.28515625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="36.5546875" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="44.88671875" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="37.88671875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="38.5546875" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="40.5546875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="240.33203125" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="132.44140625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="116.6640625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="44.33203125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="44.5546875" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="55.6640625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="129.33203125" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="155.33203125" bestFit="1" customWidth="1"/>
     <col min="61" max="61" width="43" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="73.85546875" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="47.42578125" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="46.85546875" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="39.7109375" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="43.140625" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="35.5703125" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="73.88671875" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="47.44140625" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="46.88671875" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="39.6640625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="43.109375" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="35.5546875" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="39.5546875" bestFit="1" customWidth="1"/>
     <col min="69" max="69" width="46" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="42.85546875" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="47.5703125" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="42.140625" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="132.42578125" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="128.7109375" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="47.5703125" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="39.140625" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="47.5703125" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="36.140625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="42.42578125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="40.140625" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="52.85546875" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="42.88671875" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="42.109375" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="132.44140625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="128.6640625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="39.109375" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="47.5546875" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="42.44140625" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="40.109375" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="57.88671875" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="52.88671875" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="255.6640625" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="20.5546875" bestFit="1" customWidth="1"/>
     <col min="86" max="86" width="74" bestFit="1" customWidth="1"/>
     <col min="87" max="87" width="161" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5129,7 +5129,7 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="2" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>4</v>
       </c>
@@ -5335,7 +5335,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>5</v>
       </c>
@@ -5427,7 +5427,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>6</v>
       </c>
@@ -5645,7 +5645,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>7</v>
       </c>
@@ -5737,7 +5737,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>8</v>
       </c>
@@ -5874,7 +5874,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>9</v>
       </c>
@@ -6026,7 +6026,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>10</v>
       </c>
@@ -6106,7 +6106,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>11</v>
       </c>
@@ -6186,7 +6186,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="10" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>12</v>
       </c>
@@ -6266,7 +6266,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="11" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>13</v>
       </c>
@@ -6484,7 +6484,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="12" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>14</v>
       </c>
@@ -6564,7 +6564,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="13" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>15</v>
       </c>
@@ -6713,7 +6713,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="14" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>16</v>
       </c>
@@ -6946,7 +6946,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>17</v>
       </c>
@@ -7173,7 +7173,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="16" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>18</v>
       </c>
@@ -7316,7 +7316,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>19</v>
       </c>
@@ -7408,7 +7408,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="18" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>20</v>
       </c>
@@ -7422,7 +7422,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="19" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>21</v>
       </c>
@@ -7646,7 +7646,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="20" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>22</v>
       </c>
@@ -7738,7 +7738,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="21" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>23</v>
       </c>
@@ -7968,7 +7968,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="22" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>24</v>
       </c>
@@ -8174,7 +8174,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="23" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>25</v>
       </c>
@@ -8311,7 +8311,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>26</v>
       </c>
@@ -8469,7 +8469,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>27</v>
       </c>
@@ -8606,7 +8606,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="26" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>28</v>
       </c>
@@ -8755,7 +8755,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>29</v>
       </c>
@@ -8904,7 +8904,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="28" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>30</v>
       </c>
@@ -8984,7 +8984,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="29" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>31</v>
       </c>
@@ -9193,7 +9193,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="30" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>32</v>
       </c>
@@ -9267,7 +9267,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="31" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>33</v>
       </c>
@@ -9476,7 +9476,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>34</v>
       </c>
@@ -9694,7 +9694,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>35</v>
       </c>
@@ -9900,7 +9900,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>36</v>
       </c>
@@ -10121,7 +10121,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="35" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>37</v>
       </c>
@@ -10327,7 +10327,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="36" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>38</v>
       </c>
@@ -10533,7 +10533,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="37" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>39</v>
       </c>
@@ -10739,7 +10739,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="38" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>40</v>
       </c>
@@ -10878,7 +10878,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="39" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>41</v>
       </c>
@@ -11101,7 +11101,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="40" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>42</v>
       </c>
@@ -11248,7 +11248,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="41" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>43</v>
       </c>
@@ -11343,7 +11343,7 @@
       <c r="CH41" s="1"/>
       <c r="CI41" s="1"/>
     </row>
-    <row r="42" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>44</v>
       </c>
@@ -11566,7 +11566,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="43" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>45</v>
       </c>
@@ -11713,7 +11713,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="44" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>46</v>
       </c>
@@ -11902,7 +11902,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="45" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>47</v>
       </c>
@@ -12125,7 +12125,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="46" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>48</v>
       </c>
@@ -12271,7 +12271,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="47" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>49</v>
       </c>
@@ -12494,7 +12494,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="48" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>50</v>
       </c>
@@ -12725,7 +12725,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="49" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>51</v>
       </c>
@@ -12864,7 +12864,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="50" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>52</v>
       </c>
@@ -13047,7 +13047,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="51" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>53</v>
       </c>
@@ -13276,7 +13276,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="52" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>54</v>
       </c>
@@ -13471,7 +13471,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="53" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>55</v>
       </c>
@@ -13666,7 +13666,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="54" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>56</v>
       </c>
@@ -13899,7 +13899,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="55" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>57</v>
       </c>
@@ -14094,7 +14094,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="56" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>58</v>
       </c>
@@ -14229,7 +14229,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="57" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>59</v>
       </c>
@@ -14378,7 +14378,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="58" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>60</v>
       </c>
@@ -14623,7 +14623,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="59" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>61</v>
       </c>
@@ -14860,7 +14860,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="60" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>62</v>
       </c>
@@ -15009,7 +15009,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="61" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>63</v>
       </c>
@@ -15238,7 +15238,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="62" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>64</v>
       </c>
@@ -15439,7 +15439,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="63" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>65</v>
       </c>
@@ -15634,7 +15634,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="64" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>66</v>
       </c>
@@ -15825,7 +15825,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="65" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>67</v>
       </c>
@@ -15964,7 +15964,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="66" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>68</v>
       </c>
@@ -16201,7 +16201,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="67" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>69</v>
       </c>
@@ -16348,7 +16348,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="68" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>70</v>
       </c>
@@ -16493,7 +16493,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="69" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>71</v>
       </c>
@@ -16678,7 +16678,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="70" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>72</v>
       </c>
@@ -16919,7 +16919,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="71" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>73</v>
       </c>
@@ -17162,7 +17162,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="72" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>74</v>
       </c>
@@ -17309,7 +17309,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="73" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>75</v>
       </c>
@@ -17462,7 +17462,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="74" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>76</v>
       </c>
@@ -17703,7 +17703,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="75" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>77</v>
       </c>
@@ -17942,7 +17942,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="76" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>78</v>
       </c>
@@ -18175,7 +18175,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="77" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>79</v>
       </c>
@@ -18318,7 +18318,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="78" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>80</v>
       </c>
@@ -18517,7 +18517,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="79" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>81</v>
       </c>
@@ -18662,7 +18662,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="80" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>82</v>
       </c>
@@ -18901,7 +18901,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="81" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>83</v>
       </c>
@@ -19140,7 +19140,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="82" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>84</v>
       </c>
@@ -19373,7 +19373,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="83" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>85</v>
       </c>
@@ -19512,7 +19512,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="84" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>86</v>
       </c>
@@ -19741,7 +19741,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="85" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>87</v>
       </c>
@@ -19934,7 +19934,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="86" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>88</v>
       </c>
@@ -20073,7 +20073,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="87" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>89</v>
       </c>
@@ -20208,7 +20208,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="88" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>90</v>
       </c>
@@ -20461,7 +20461,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="89" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>91</v>
       </c>
@@ -20596,7 +20596,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="90" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>92</v>
       </c>
@@ -20735,7 +20735,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="91" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>93</v>
       </c>
@@ -20922,7 +20922,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="92" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>94</v>
       </c>
@@ -21061,7 +21061,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="93" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>95</v>
       </c>
@@ -21198,7 +21198,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="94" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>96</v>
       </c>
@@ -21345,7 +21345,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="95" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>97</v>
       </c>
@@ -21484,7 +21484,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="96" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>98</v>
       </c>
@@ -21623,7 +21623,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="97" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>99</v>
       </c>
@@ -21852,7 +21852,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="98" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>100</v>
       </c>
@@ -21991,7 +21991,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="99" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>101</v>
       </c>
@@ -22170,7 +22170,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="100" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>102</v>
       </c>
@@ -22355,7 +22355,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="101" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>103</v>
       </c>
@@ -22534,7 +22534,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="102" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>104</v>
       </c>
@@ -22713,7 +22713,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="103" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>105</v>
       </c>
@@ -22898,7 +22898,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="104" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>106</v>
       </c>
@@ -23037,7 +23037,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="105" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>107</v>
       </c>
@@ -23182,7 +23182,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="106" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>108</v>
       </c>
@@ -23419,7 +23419,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="107" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>109</v>
       </c>
@@ -23656,7 +23656,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="108" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>110</v>
       </c>
@@ -23885,7 +23885,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="109" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>111</v>
       </c>
@@ -24024,7 +24024,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="110" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>112</v>
       </c>
@@ -24207,7 +24207,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="111" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>113</v>
       </c>
@@ -24354,7 +24354,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="112" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>114</v>
       </c>
@@ -24493,7 +24493,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="113" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>115</v>
       </c>
@@ -24632,7 +24632,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="114" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>116</v>
       </c>
@@ -24771,7 +24771,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="115" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>117</v>
       </c>
@@ -24918,7 +24918,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="116" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>118</v>
       </c>
@@ -25067,7 +25067,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="117" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>119</v>
       </c>
@@ -25258,7 +25258,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="118" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>120</v>
       </c>
@@ -25445,7 +25445,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="119" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>121</v>
       </c>
@@ -25682,7 +25682,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="120" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>122</v>
       </c>
@@ -25873,7 +25873,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="121" spans="1:87" ht="30" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:87" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>123</v>
       </c>
@@ -26104,7 +26104,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="122" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>124</v>
       </c>
@@ -26335,7 +26335,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="123" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>125</v>
       </c>
@@ -26570,7 +26570,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="124" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>126</v>
       </c>
@@ -26801,7 +26801,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="125" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>127</v>
       </c>
@@ -27032,7 +27032,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="126" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>128</v>
       </c>
@@ -27269,7 +27269,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="127" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>129</v>
       </c>
@@ -27416,7 +27416,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="128" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>130</v>
       </c>
@@ -27599,7 +27599,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="129" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>131</v>
       </c>
@@ -27782,7 +27782,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="130" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>132</v>
       </c>
@@ -28019,7 +28019,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="131" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>133</v>
       </c>
@@ -28202,7 +28202,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="132" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>134</v>
       </c>
@@ -28349,7 +28349,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="133" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>135</v>
       </c>
@@ -28486,7 +28486,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="134" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>136</v>
       </c>
@@ -28725,7 +28725,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="135" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>137</v>
       </c>
@@ -28908,7 +28908,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="136" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>138</v>
       </c>
@@ -29137,7 +29137,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="137" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>139</v>
       </c>
@@ -29276,7 +29276,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="138" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>140</v>
       </c>
@@ -29413,7 +29413,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="139" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>141</v>
       </c>
@@ -29550,7 +29550,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="140" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>142</v>
       </c>
@@ -29685,7 +29685,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="141" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>143</v>
       </c>
@@ -29820,7 +29820,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="142" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>144</v>
       </c>
@@ -29959,7 +29959,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="143" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>145</v>
       </c>
@@ -30188,7 +30188,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="144" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>146</v>
       </c>
@@ -30327,7 +30327,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="145" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>147</v>
       </c>
@@ -30556,7 +30556,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="146" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>148</v>
       </c>
@@ -30739,7 +30739,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="147" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>149</v>
       </c>
@@ -30922,7 +30922,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="148" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>150</v>
       </c>
@@ -31061,7 +31061,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="149" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>151</v>
       </c>
@@ -31208,7 +31208,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="150" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>152</v>
       </c>
@@ -31449,7 +31449,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="151" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>153</v>
       </c>
@@ -31688,7 +31688,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="152" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>154</v>
       </c>
@@ -31917,7 +31917,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="153" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>155</v>
       </c>
@@ -32056,7 +32056,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="154" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>156</v>
       </c>
@@ -32203,7 +32203,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="155" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>157</v>
       </c>
@@ -32438,7 +32438,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="156" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>158</v>
       </c>
@@ -32577,7 +32577,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="157" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>159</v>
       </c>
@@ -32806,7 +32806,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="158" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>160</v>
       </c>
@@ -33035,7 +33035,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="159" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>161</v>
       </c>
@@ -33272,7 +33272,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="160" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>162</v>
       </c>
@@ -33419,7 +33419,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="161" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>163</v>
       </c>
@@ -33566,7 +33566,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="162" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>164</v>
       </c>
@@ -33799,7 +33799,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="163" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>165</v>
       </c>
@@ -33984,7 +33984,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="164" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>166</v>
       </c>
@@ -34167,7 +34167,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="165" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>167</v>
       </c>
@@ -34306,7 +34306,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="166" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>168</v>
       </c>
@@ -34445,7 +34445,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="167" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>169</v>
       </c>
@@ -34672,7 +34672,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="168" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>170</v>
       </c>
@@ -34875,7 +34875,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="169" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>171</v>
       </c>
@@ -35070,7 +35070,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="170" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>172</v>
       </c>
@@ -35165,7 +35165,7 @@
       <c r="CH170" s="1"/>
       <c r="CI170" s="1"/>
     </row>
-    <row r="171" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>173</v>
       </c>
@@ -35408,7 +35408,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="172" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>174</v>
       </c>
@@ -35547,7 +35547,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="173" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>175</v>
       </c>
@@ -35686,7 +35686,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="174" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>176</v>
       </c>
@@ -35917,7 +35917,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="175" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>177</v>
       </c>
@@ -36146,7 +36146,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="176" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>178</v>
       </c>
@@ -36283,7 +36283,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="177" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>179</v>
       </c>
@@ -36430,7 +36430,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="178" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>180</v>
       </c>
@@ -36665,7 +36665,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="179" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>181</v>
       </c>
@@ -36804,7 +36804,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="180" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>182</v>
       </c>
@@ -36951,7 +36951,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="181" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>183</v>
       </c>
@@ -37094,7 +37094,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="182" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>184</v>
       </c>
@@ -37233,7 +37233,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="183" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>185</v>
       </c>
@@ -37372,7 +37372,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="184" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>186</v>
       </c>
@@ -37551,7 +37551,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="185" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>187</v>
       </c>
@@ -37736,7 +37736,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="186" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>188</v>
       </c>
@@ -37965,7 +37965,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="187" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>189</v>
       </c>
@@ -38150,7 +38150,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="188" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>190</v>
       </c>
@@ -38377,7 +38377,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="189" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>191</v>
       </c>
@@ -38516,7 +38516,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="190" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>192</v>
       </c>
@@ -38745,7 +38745,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="191" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>193</v>
       </c>
@@ -38884,7 +38884,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="192" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>194</v>
       </c>
@@ -39031,7 +39031,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="193" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>195</v>
       </c>
@@ -39214,7 +39214,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="194" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>196</v>
       </c>
@@ -39353,7 +39353,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="195" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>197</v>
       </c>
@@ -39536,7 +39536,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="196" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>198</v>
       </c>
@@ -39785,7 +39785,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="197" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>199</v>
       </c>
@@ -40016,7 +40016,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="198" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>200</v>
       </c>
@@ -40245,7 +40245,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="199" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>201</v>
       </c>
@@ -40430,7 +40430,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="200" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>202</v>
       </c>
@@ -40569,7 +40569,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="201" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>203</v>
       </c>
@@ -40822,7 +40822,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="202" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>204</v>
       </c>
@@ -41017,7 +41017,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="203" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>205</v>
       </c>
@@ -41198,7 +41198,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="204" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>206</v>
       </c>
@@ -41389,7 +41389,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="205" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>207</v>
       </c>
@@ -41626,7 +41626,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="206" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>208</v>
       </c>
@@ -41855,7 +41855,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="207" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>209</v>
       </c>
@@ -42008,7 +42008,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="208" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>210</v>
       </c>
@@ -42161,7 +42161,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="209" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>211</v>
       </c>
@@ -42372,7 +42372,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="210" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>212</v>
       </c>
@@ -42555,7 +42555,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="211" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>213</v>
       </c>
@@ -42740,7 +42740,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="212" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>214</v>
       </c>
@@ -42969,7 +42969,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="213" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>215</v>
       </c>
@@ -43158,7 +43158,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="214" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>216</v>
       </c>
@@ -43297,7 +43297,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="215" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>217</v>
       </c>
@@ -43478,7 +43478,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="216" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>218</v>
       </c>
@@ -43707,7 +43707,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="217" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>219</v>
       </c>
@@ -43856,7 +43856,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="218" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>220</v>
       </c>
@@ -43999,7 +43999,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="219" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>221</v>
       </c>
@@ -44182,7 +44182,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="220" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>222</v>
       </c>
@@ -44367,7 +44367,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="221" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>223</v>
       </c>
@@ -44510,7 +44510,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="222" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>224</v>
       </c>
@@ -44605,7 +44605,7 @@
       <c r="CH222" s="1"/>
       <c r="CI222" s="1"/>
     </row>
-    <row r="223" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>225</v>
       </c>
@@ -44788,7 +44788,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="224" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>226</v>
       </c>
@@ -45037,7 +45037,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="225" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>227</v>
       </c>
@@ -45280,7 +45280,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="226" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>228</v>
       </c>
@@ -45469,7 +45469,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="227" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>229</v>
       </c>
@@ -45608,7 +45608,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="228" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>230</v>
       </c>
@@ -45791,7 +45791,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="229" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>231</v>
       </c>
@@ -45978,7 +45978,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="230" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>232</v>
       </c>
@@ -46117,7 +46117,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="231" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>233</v>
       </c>
@@ -46300,7 +46300,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="232" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>234</v>
       </c>
@@ -46453,7 +46453,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="233" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>235</v>
       </c>
@@ -46636,7 +46636,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="234" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>236</v>
       </c>
@@ -46875,7 +46875,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="235" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>237</v>
       </c>
@@ -47036,7 +47036,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="236" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>238</v>
       </c>
@@ -47265,7 +47265,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="237" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>239</v>
       </c>
@@ -47404,7 +47404,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="238" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>240</v>
       </c>
@@ -47641,7 +47641,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="239" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>241</v>
       </c>
@@ -47878,7 +47878,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="240" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>242</v>
       </c>
@@ -48125,7 +48125,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="241" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>243</v>
       </c>
@@ -48362,7 +48362,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="242" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>244</v>
       </c>
@@ -48591,7 +48591,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="243" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>245</v>
       </c>
@@ -48730,7 +48730,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="244" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>246</v>
       </c>
@@ -48965,7 +48965,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="245" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>247</v>
       </c>
@@ -49112,7 +49112,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="246" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>248</v>
       </c>
@@ -49347,7 +49347,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="247" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>249</v>
       </c>
@@ -49592,7 +49592,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="248" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>250</v>
       </c>
@@ -49731,7 +49731,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="249" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>251</v>
       </c>
@@ -49980,7 +49980,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="250" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>252</v>
       </c>
@@ -50221,7 +50221,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="251" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>253</v>
       </c>
@@ -50374,7 +50374,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="252" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>254</v>
       </c>
@@ -50521,7 +50521,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="253" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>255</v>
       </c>
@@ -50750,7 +50750,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="254" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>256</v>
       </c>
@@ -50979,7 +50979,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="255" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>257</v>
       </c>
@@ -51126,7 +51126,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="256" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>258</v>
       </c>
@@ -51265,7 +51265,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="257" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>259</v>
       </c>
@@ -51410,7 +51410,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="258" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>260</v>
       </c>
@@ -51549,7 +51549,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="259" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>261</v>
       </c>
@@ -51738,7 +51738,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="260" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>262</v>
       </c>
@@ -51979,7 +51979,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="261" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>263</v>
       </c>
@@ -52208,7 +52208,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="262" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>264</v>
       </c>
@@ -52419,7 +52419,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="263" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>265</v>
       </c>
@@ -52558,7 +52558,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="264" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>266</v>
       </c>
@@ -52701,7 +52701,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="265" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>267</v>
       </c>
@@ -52930,7 +52930,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="266" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>268</v>
       </c>
@@ -53171,7 +53171,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="267" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>269</v>
       </c>
@@ -53358,7 +53358,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="268" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>270</v>
       </c>
@@ -53585,7 +53585,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="269" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>271</v>
       </c>
@@ -53770,7 +53770,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="270" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>272</v>
       </c>
@@ -53915,7 +53915,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="271" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>273</v>
       </c>
@@ -54062,7 +54062,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="272" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>274</v>
       </c>
@@ -54305,7 +54305,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="273" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>275</v>
       </c>
@@ -54534,7 +54534,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="274" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>276</v>
       </c>
@@ -54717,7 +54717,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="275" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>277</v>
       </c>
@@ -54942,7 +54942,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="276" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>278</v>
       </c>
@@ -55089,7 +55089,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="277" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>279</v>
       </c>
@@ -55314,7 +55314,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="278" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>280</v>
       </c>
@@ -55539,7 +55539,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="279" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>281</v>
       </c>
@@ -55684,7 +55684,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="280" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>282</v>
       </c>
@@ -55869,7 +55869,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="281" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>283</v>
       </c>
@@ -56098,7 +56098,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="282" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>284</v>
       </c>
@@ -56235,7 +56235,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="283" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>285</v>
       </c>
@@ -56418,7 +56418,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="284" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>286</v>
       </c>
@@ -56609,7 +56609,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="285" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>287</v>
       </c>
@@ -56746,7 +56746,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="286" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>288</v>
       </c>
@@ -56975,7 +56975,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="287" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>289</v>
       </c>
@@ -57166,7 +57166,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="288" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>290</v>
       </c>
@@ -57319,7 +57319,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="289" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>291</v>
       </c>
@@ -57544,7 +57544,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="290" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>292</v>
       </c>
@@ -57769,7 +57769,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="291" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>293</v>
       </c>
@@ -57908,7 +57908,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="292" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>294</v>
       </c>
@@ -58047,7 +58047,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="293" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>295</v>
       </c>
@@ -58296,7 +58296,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="294" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>296</v>
       </c>
@@ -58435,7 +58435,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="295" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>297</v>
       </c>
@@ -58622,7 +58622,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="296" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>298</v>
       </c>
@@ -58859,7 +58859,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="297" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>299</v>
       </c>
@@ -59042,7 +59042,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="298" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>300</v>
       </c>
@@ -59271,7 +59271,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="299" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>301</v>
       </c>
@@ -59418,7 +59418,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="300" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>302</v>
       </c>
@@ -59649,7 +59649,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="301" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>303</v>
       </c>
@@ -59838,7 +59838,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="302" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>304</v>
       </c>
@@ -60075,7 +60075,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="303" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>305</v>
       </c>
@@ -60304,7 +60304,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="304" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>306</v>
       </c>
@@ -60451,7 +60451,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="305" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>307</v>
       </c>
@@ -60634,7 +60634,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="306" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>308</v>
       </c>
@@ -60813,7 +60813,7 @@
         <v>886</v>
       </c>
     </row>
-    <row r="307" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>309</v>
       </c>
@@ -61064,7 +61064,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="308" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>310</v>
       </c>
@@ -61207,7 +61207,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="309" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>311</v>
       </c>
@@ -61398,7 +61398,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="310" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>312</v>
       </c>
@@ -61537,7 +61537,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="311" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>313</v>
       </c>
@@ -61632,7 +61632,7 @@
       <c r="CH311" s="1"/>
       <c r="CI311" s="1"/>
     </row>
-    <row r="312" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>314</v>
       </c>
@@ -61771,7 +61771,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="313" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>315</v>
       </c>
@@ -61954,7 +61954,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="314" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>316</v>
       </c>
@@ -62093,7 +62093,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="315" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>317</v>
       </c>
@@ -62240,7 +62240,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="316" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>318</v>
       </c>
@@ -62469,7 +62469,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="317" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>319</v>
       </c>
@@ -62728,7 +62728,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="318" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>320</v>
       </c>
@@ -62875,7 +62875,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="319" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>321</v>
       </c>
@@ -63014,7 +63014,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="320" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>322</v>
       </c>
@@ -63173,7 +63173,7 @@
         <v>919</v>
       </c>
     </row>
-    <row r="321" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>323</v>
       </c>
@@ -63376,7 +63376,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="322" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>324</v>
       </c>
@@ -63613,7 +63613,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="323" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>325</v>
       </c>
@@ -63800,7 +63800,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="324" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>326</v>
       </c>
@@ -64037,7 +64037,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="325" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>327</v>
       </c>
@@ -64266,7 +64266,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="326" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>328</v>
       </c>
@@ -64495,7 +64495,7 @@
         <v>932</v>
       </c>
     </row>
-    <row r="327" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>329</v>
       </c>
@@ -64748,7 +64748,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="328" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>330</v>
       </c>
@@ -64895,7 +64895,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="329" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>331</v>
       </c>
@@ -65042,7 +65042,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="330" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>332</v>
       </c>
@@ -65229,7 +65229,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="331" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>333</v>
       </c>
@@ -65376,7 +65376,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="332" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>334</v>
       </c>
@@ -65529,7 +65529,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="333" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>335</v>
       </c>
@@ -65766,7 +65766,7 @@
         <v>950</v>
       </c>
     </row>
-    <row r="334" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>336</v>
       </c>
@@ -66001,7 +66001,7 @@
         <v>958</v>
       </c>
     </row>
-    <row r="335" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>337</v>
       </c>
@@ -66248,7 +66248,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="336" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>338</v>
       </c>
@@ -66477,7 +66477,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="337" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>339</v>
       </c>
@@ -66670,7 +66670,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="338" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>340</v>
       </c>
@@ -66907,7 +66907,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="339" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>341</v>
       </c>
@@ -67052,7 +67052,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="340" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>342</v>
       </c>
@@ -67247,7 +67247,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="341" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>343</v>
       </c>
@@ -67394,7 +67394,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="342" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A342">
         <v>344</v>
       </c>
@@ -67541,7 +67541,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="343" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>345</v>
       </c>
@@ -67772,7 +67772,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="344" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A344">
         <v>346</v>
       </c>
@@ -67965,7 +67965,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="345" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A345">
         <v>347</v>
       </c>
@@ -68166,7 +68166,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="346" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A346">
         <v>348</v>
       </c>
@@ -68305,7 +68305,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="347" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A347">
         <v>349</v>
       </c>
@@ -68496,7 +68496,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="348" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A348">
         <v>350</v>
       </c>
@@ -68733,7 +68733,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="349" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>351</v>
       </c>
@@ -68962,7 +68962,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="350" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A350">
         <v>352</v>
       </c>
@@ -69155,7 +69155,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="351" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>353</v>
       </c>
@@ -69390,7 +69390,7 @@
         <v>725</v>
       </c>
     </row>
-    <row r="352" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A352">
         <v>354</v>
       </c>
@@ -69619,7 +69619,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="353" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A353">
         <v>355</v>
       </c>
@@ -69874,7 +69874,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="354" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A354">
         <v>356</v>
       </c>
@@ -70103,7 +70103,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="355" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A355">
         <v>357</v>
       </c>
@@ -70288,7 +70288,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="356" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A356">
         <v>358</v>
       </c>
@@ -70469,7 +70469,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="357" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A357">
         <v>359</v>
       </c>
@@ -70616,7 +70616,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="358" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A358">
         <v>360</v>
       </c>
@@ -70755,7 +70755,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="359" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A359">
         <v>361</v>
       </c>
@@ -70890,7 +70890,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="360" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A360">
         <v>362</v>
       </c>
@@ -71035,7 +71035,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="361" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A361">
         <v>363</v>
       </c>
@@ -71174,7 +71174,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="362" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A362">
         <v>364</v>
       </c>
@@ -71367,7 +71367,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="363" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A363">
         <v>365</v>
       </c>
@@ -71596,7 +71596,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="364" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A364">
         <v>366</v>
       </c>
@@ -71789,7 +71789,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="365" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A365">
         <v>367</v>
       </c>
@@ -71936,7 +71936,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="366" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A366">
         <v>368</v>
       </c>
@@ -72167,7 +72167,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="367" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A367">
         <v>369</v>
       </c>
@@ -72306,7 +72306,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="368" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A368">
         <v>370</v>
       </c>
@@ -72511,7 +72511,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="369" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A369">
         <v>371</v>
       </c>
@@ -72742,7 +72742,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="370" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A370">
         <v>372</v>
       </c>
@@ -72881,7 +72881,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="371" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A371">
         <v>373</v>
       </c>
@@ -73120,7 +73120,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="372" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A372">
         <v>374</v>
       </c>
@@ -73267,7 +73267,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="373" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A373">
         <v>375</v>
       </c>
@@ -73412,7 +73412,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="374" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A374">
         <v>376</v>
       </c>
@@ -73645,7 +73645,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="375" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A375">
         <v>377</v>
       </c>
@@ -73874,7 +73874,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="376" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A376">
         <v>378</v>
       </c>
@@ -74103,7 +74103,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="377" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A377">
         <v>379</v>
       </c>
@@ -74238,7 +74238,7 @@
         <v>1029</v>
       </c>
     </row>
-    <row r="378" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A378">
         <v>380</v>
       </c>
@@ -74377,7 +74377,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="379" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A379">
         <v>381</v>
       </c>
@@ -74514,7 +74514,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="380" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A380">
         <v>382</v>
       </c>
@@ -74751,7 +74751,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="381" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A381">
         <v>383</v>
       </c>
@@ -74982,7 +74982,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="382" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A382">
         <v>384</v>
       </c>
@@ -75217,7 +75217,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="383" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A383">
         <v>385</v>
       </c>
@@ -75360,7 +75360,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="384" spans="1:87" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:87" x14ac:dyDescent="0.3">
       <c r="A384">
         <v>386</v>
       </c>

</xml_diff>